<commit_message>
Problem: substring with concatenation
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="319">
   <si>
     <t>date</t>
   </si>
@@ -967,6 +967,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-substring-without-repeating-characters/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">substring with concatentation of all words</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/substring-with-concatenation-of-all-words/</t>
   </si>
 </sst>
 </file>
@@ -3258,6 +3264,17 @@
         <v>316</v>
       </c>
     </row>
+    <row r="159" ht="14.25">
+      <c r="A159" s="1">
+        <v>46150</v>
+      </c>
+      <c r="B159" t="s">
+        <v>317</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3416,6 +3433,7 @@
     <hyperlink r:id="rId154" ref="C156"/>
     <hyperlink r:id="rId155" ref="C157"/>
     <hyperlink r:id="rId156" ref="C158"/>
+    <hyperlink r:id="rId157" ref="C159"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: min. window substring
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="321">
   <si>
     <t>date</t>
   </si>
@@ -973,6 +973,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/substring-with-concatenation-of-all-words/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min win substr.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-window-substring/</t>
   </si>
 </sst>
 </file>
@@ -3275,6 +3281,17 @@
         <v>318</v>
       </c>
     </row>
+    <row r="160" ht="14.25">
+      <c r="A160" s="1">
+        <v>46150</v>
+      </c>
+      <c r="B160" t="s">
+        <v>319</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3434,6 +3451,7 @@
     <hyperlink r:id="rId155" ref="C157"/>
     <hyperlink r:id="rId156" ref="C158"/>
     <hyperlink r:id="rId157" ref="C159"/>
+    <hyperlink r:id="rId158" ref="C160"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: two sum II - Input array is sorted
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="329">
   <si>
     <t>date</t>
   </si>
@@ -997,6 +997,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/number-of-matching-subsequences/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">two sum II - Input Array is Sorted</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/</t>
   </si>
 </sst>
 </file>
@@ -3343,6 +3349,17 @@
         <v>326</v>
       </c>
     </row>
+    <row r="164" ht="14.25">
+      <c r="A164" s="1">
+        <v>46152</v>
+      </c>
+      <c r="B164" t="s">
+        <v>327</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3506,6 +3523,7 @@
     <hyperlink r:id="rId159" ref="C161"/>
     <hyperlink r:id="rId160" ref="C162"/>
     <hyperlink r:id="rId161" ref="C163"/>
+    <hyperlink r:id="rId162" ref="C164"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: container with most water
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="331">
   <si>
     <t>date</t>
   </si>
@@ -1003,6 +1003,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">container with most water</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/container-with-most-water/</t>
   </si>
 </sst>
 </file>
@@ -3360,6 +3366,17 @@
         <v>328</v>
       </c>
     </row>
+    <row r="165" ht="14.25">
+      <c r="A165" s="1">
+        <v>46152</v>
+      </c>
+      <c r="B165" t="s">
+        <v>329</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3524,6 +3541,7 @@
     <hyperlink r:id="rId160" ref="C162"/>
     <hyperlink r:id="rId161" ref="C163"/>
     <hyperlink r:id="rId162" ref="C164"/>
+    <hyperlink r:id="rId163" ref="C165"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: merge 2 sorted arrays
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="336">
   <si>
     <t>date</t>
   </si>
@@ -1015,6 +1015,15 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/3sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">merge sorted array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">merge without extra space</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/merge-two-sorted-arrays-1587115620/1</t>
   </si>
 </sst>
 </file>
@@ -3394,6 +3403,28 @@
         <v>332</v>
       </c>
     </row>
+    <row r="167" ht="14.25">
+      <c r="A167" s="1">
+        <v>46153</v>
+      </c>
+      <c r="B167" t="s">
+        <v>333</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="168" ht="14.25">
+      <c r="A168" s="1">
+        <v>46153</v>
+      </c>
+      <c r="B168" t="s">
+        <v>334</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3560,6 +3591,8 @@
     <hyperlink r:id="rId162" ref="C164"/>
     <hyperlink r:id="rId163" ref="C165"/>
     <hyperlink r:id="rId164" ref="C166"/>
+    <hyperlink r:id="rId15" ref="C167"/>
+    <hyperlink r:id="rId165" ref="C168"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: remove duplicates from sorted array and remove element
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="339">
   <si>
     <t>date</t>
   </si>
@@ -1017,13 +1017,22 @@
     <t>https://leetcode.com/problems/3sum/</t>
   </si>
   <si>
-    <t xml:space="preserve">merge sorted array</t>
-  </si>
-  <si>
     <t xml:space="preserve">merge without extra space</t>
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/merge-two-sorted-arrays-1587115620/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove element</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-element/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove duplicates from sorted array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-duplicates-from-sorted-array/</t>
   </si>
 </sst>
 </file>
@@ -3411,7 +3420,7 @@
         <v>333</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>34</v>
+        <v>334</v>
       </c>
     </row>
     <row r="168" ht="14.25">
@@ -3419,10 +3428,21 @@
         <v>46153</v>
       </c>
       <c r="B168" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
+      </c>
+    </row>
+    <row r="169" ht="14.25">
+      <c r="A169" s="1">
+        <v>46153</v>
+      </c>
+      <c r="B169" t="s">
+        <v>337</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -3591,8 +3611,9 @@
     <hyperlink r:id="rId162" ref="C164"/>
     <hyperlink r:id="rId163" ref="C165"/>
     <hyperlink r:id="rId164" ref="C166"/>
-    <hyperlink r:id="rId15" ref="C167"/>
-    <hyperlink r:id="rId165" ref="C168"/>
+    <hyperlink r:id="rId165" ref="C167"/>
+    <hyperlink r:id="rId166" ref="C168"/>
+    <hyperlink r:id="rId167" ref="C169"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: jump game II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="347">
   <si>
     <t>date</t>
   </si>
@@ -1051,6 +1051,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/jump-game/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jump game II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/jump-game-ii/</t>
   </si>
 </sst>
 </file>
@@ -3497,6 +3503,17 @@
         <v>344</v>
       </c>
     </row>
+    <row r="173" ht="14.25">
+      <c r="A173" s="1">
+        <v>46155</v>
+      </c>
+      <c r="B173" t="s">
+        <v>345</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3669,6 +3686,7 @@
     <hyperlink r:id="rId168" ref="C170"/>
     <hyperlink r:id="rId169" ref="C171"/>
     <hyperlink r:id="rId170" ref="C172"/>
+    <hyperlink r:id="rId171" ref="C173"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: insert delete random O(1)
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="351">
   <si>
     <t>date</t>
   </si>
@@ -1063,6 +1063,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/h-index/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insert Delete Random - O(1)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/insert-delete-getrandom-o1/</t>
   </si>
 </sst>
 </file>
@@ -3531,6 +3537,17 @@
         <v>348</v>
       </c>
     </row>
+    <row r="175" ht="14.25">
+      <c r="A175" s="1">
+        <v>46157</v>
+      </c>
+      <c r="B175" t="s">
+        <v>349</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3705,6 +3722,7 @@
     <hyperlink r:id="rId170" ref="C172"/>
     <hyperlink r:id="rId171" ref="C173"/>
     <hyperlink r:id="rId172" ref="C174"/>
+    <hyperlink r:id="rId173" ref="C175"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: product of array except self
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="353">
   <si>
     <t>date</t>
   </si>
@@ -1069,6 +1069,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/insert-delete-getrandom-o1/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product of array except self</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/product-of-array-except-self/</t>
   </si>
 </sst>
 </file>
@@ -3548,6 +3554,17 @@
         <v>350</v>
       </c>
     </row>
+    <row r="176" ht="14.25">
+      <c r="A176" s="1">
+        <v>46158</v>
+      </c>
+      <c r="B176" t="s">
+        <v>351</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>352</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3723,6 +3740,7 @@
     <hyperlink r:id="rId171" ref="C173"/>
     <hyperlink r:id="rId172" ref="C174"/>
     <hyperlink r:id="rId173" ref="C175"/>
+    <hyperlink r:id="rId174" ref="C176"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: trapping rain water
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="359">
   <si>
     <t>date</t>
   </si>
@@ -1087,6 +1087,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/candy/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trapping Rain Water</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/trapping-rain-water/</t>
   </si>
 </sst>
 </file>
@@ -3599,6 +3605,17 @@
         <v>356</v>
       </c>
     </row>
+    <row r="179" ht="14.25">
+      <c r="A179" s="1">
+        <v>46159</v>
+      </c>
+      <c r="B179" t="s">
+        <v>357</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3777,6 +3794,7 @@
     <hyperlink r:id="rId174" ref="C176"/>
     <hyperlink r:id="rId175" ref="C177"/>
     <hyperlink r:id="rId176" ref="C178"/>
+    <hyperlink r:id="rId177" ref="C179"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: roman to integer
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="361">
   <si>
     <t>date</t>
   </si>
@@ -1093,6 +1093,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/trapping-rain-water/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roman to Integer</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/roman-to-integer/</t>
   </si>
 </sst>
 </file>
@@ -3616,6 +3622,17 @@
         <v>358</v>
       </c>
     </row>
+    <row r="180" ht="14.25">
+      <c r="A180" s="1">
+        <v>46160</v>
+      </c>
+      <c r="B180" t="s">
+        <v>359</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3795,6 +3812,7 @@
     <hyperlink r:id="rId175" ref="C177"/>
     <hyperlink r:id="rId176" ref="C178"/>
     <hyperlink r:id="rId177" ref="C179"/>
+    <hyperlink r:id="rId178" ref="C180"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: integer to roman
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="363">
   <si>
     <t>date</t>
   </si>
@@ -1099,6 +1099,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/roman-to-integer/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integer to Roman</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/integer-to-roman/</t>
   </si>
 </sst>
 </file>
@@ -1139,7 +1145,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -1151,6 +1157,7 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3633,6 +3640,17 @@
         <v>360</v>
       </c>
     </row>
+    <row r="181" ht="14.25">
+      <c r="A181" s="7">
+        <v>46160</v>
+      </c>
+      <c r="B181" t="s">
+        <v>361</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3813,6 +3831,7 @@
     <hyperlink r:id="rId176" ref="C178"/>
     <hyperlink r:id="rId177" ref="C179"/>
     <hyperlink r:id="rId178" ref="C180"/>
+    <hyperlink r:id="rId179" ref="C181"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: length of last word in a string
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="365">
   <si>
     <t>date</t>
   </si>
@@ -1105,6 +1105,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/integer-to-roman/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Length of last word</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/length-of-last-word/</t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1151,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -1157,7 +1163,6 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3641,7 +3646,7 @@
       </c>
     </row>
     <row r="181" ht="14.25">
-      <c r="A181" s="7">
+      <c r="A181" s="1">
         <v>46160</v>
       </c>
       <c r="B181" t="s">
@@ -3649,6 +3654,17 @@
       </c>
       <c r="C181" s="2" t="s">
         <v>362</v>
+      </c>
+    </row>
+    <row r="182" ht="14.25">
+      <c r="A182" s="1">
+        <v>46161</v>
+      </c>
+      <c r="B182" t="s">
+        <v>363</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -3832,6 +3848,7 @@
     <hyperlink r:id="rId177" ref="C179"/>
     <hyperlink r:id="rId178" ref="C180"/>
     <hyperlink r:id="rId179" ref="C181"/>
+    <hyperlink r:id="rId180" ref="C182"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: longest common prefix
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="367">
   <si>
     <t>date</t>
   </si>
@@ -1111,6 +1111,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/length-of-last-word/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">longest common prefix</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-common-prefix/</t>
   </si>
 </sst>
 </file>
@@ -3667,6 +3673,17 @@
         <v>364</v>
       </c>
     </row>
+    <row r="183" ht="14.25">
+      <c r="A183" s="1">
+        <v>46161</v>
+      </c>
+      <c r="B183" t="s">
+        <v>365</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3849,6 +3866,7 @@
     <hyperlink r:id="rId178" ref="C180"/>
     <hyperlink r:id="rId179" ref="C181"/>
     <hyperlink r:id="rId180" ref="C182"/>
+    <hyperlink r:id="rId181" ref="C183"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: find the idx. of the first occurance in a string
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="373">
   <si>
     <t>date</t>
   </si>
@@ -1129,6 +1129,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/zigzag-conversion/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">find the idx of the first occurance of the string</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-the-index-of-the-first-occurrence-in-a-string/</t>
   </si>
 </sst>
 </file>
@@ -3718,6 +3724,17 @@
         <v>370</v>
       </c>
     </row>
+    <row r="186" ht="14.25">
+      <c r="A186" s="1">
+        <v>46163</v>
+      </c>
+      <c r="B186" t="s">
+        <v>371</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3903,6 +3920,7 @@
     <hyperlink r:id="rId181" ref="C183"/>
     <hyperlink r:id="rId182" ref="C184"/>
     <hyperlink r:id="rId183" ref="C185"/>
+    <hyperlink r:id="rId184" ref="C186"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: frog jump with k distances
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="384">
   <si>
     <t>date</t>
   </si>
@@ -1162,6 +1162,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/geek-jump/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">frog jump with k distances</t>
+  </si>
+  <si>
+    <t>https://takeuforward.org/plus/dsa/problems/frog-jump-with-k-distances</t>
   </si>
 </sst>
 </file>
@@ -3813,6 +3819,17 @@
         <v>381</v>
       </c>
     </row>
+    <row r="192" ht="14.25">
+      <c r="A192" s="1">
+        <v>46169</v>
+      </c>
+      <c r="B192" t="s">
+        <v>382</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4003,6 +4020,7 @@
     <hyperlink r:id="rId186" ref="C189"/>
     <hyperlink r:id="rId187" ref="C190"/>
     <hyperlink r:id="rId188" ref="C191"/>
+    <hyperlink r:id="rId189" ref="C192"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: House Robber II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="388">
   <si>
     <t>date</t>
   </si>
@@ -1174,6 +1174,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/reorganize-string/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">House Robber II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/house-robber-ii/</t>
   </si>
 </sst>
 </file>
@@ -3847,6 +3853,17 @@
         <v>385</v>
       </c>
     </row>
+    <row r="194" ht="14.25">
+      <c r="A194" s="1">
+        <v>46171</v>
+      </c>
+      <c r="B194" t="s">
+        <v>386</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4039,6 +4056,7 @@
     <hyperlink r:id="rId188" ref="C191"/>
     <hyperlink r:id="rId189" ref="C192"/>
     <hyperlink r:id="rId190" ref="C193"/>
+    <hyperlink r:id="rId191" ref="C194"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: minimum cost to connect all ropes
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="390">
   <si>
     <t>date</t>
   </si>
@@ -1180,6 +1180,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/house-robber-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min. cost of ropes </t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/minimum-cost-of-ropes-1587115620/1</t>
   </si>
 </sst>
 </file>
@@ -3864,6 +3870,17 @@
         <v>387</v>
       </c>
     </row>
+    <row r="195" ht="14.25">
+      <c r="A195" s="1">
+        <v>46172</v>
+      </c>
+      <c r="B195" t="s">
+        <v>388</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4057,6 +4074,7 @@
     <hyperlink r:id="rId189" ref="C192"/>
     <hyperlink r:id="rId190" ref="C193"/>
     <hyperlink r:id="rId191" ref="C194"/>
+    <hyperlink r:id="rId192" ref="C195"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: sliding win. max.
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="394">
   <si>
     <t>date</t>
   </si>
@@ -1192,6 +1192,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/geeks-training/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sliding window maximum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sliding-window-maximum/</t>
   </si>
 </sst>
 </file>
@@ -3898,6 +3904,17 @@
         <v>391</v>
       </c>
     </row>
+    <row r="197" ht="14.25">
+      <c r="A197" s="1">
+        <v>46173</v>
+      </c>
+      <c r="B197" t="s">
+        <v>392</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>393</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4093,6 +4110,7 @@
     <hyperlink r:id="rId191" ref="C194"/>
     <hyperlink r:id="rId192" ref="C195"/>
     <hyperlink r:id="rId193" ref="C196"/>
+    <hyperlink r:id="rId194" ref="C197"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: top k frequent words
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="398">
   <si>
     <t>date</t>
   </si>
@@ -1204,6 +1204,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/unique-paths/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top k frequent words</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/top-k-frequent-words/</t>
   </si>
 </sst>
 </file>
@@ -3932,6 +3938,17 @@
         <v>395</v>
       </c>
     </row>
+    <row r="199" ht="14.25">
+      <c r="A199" s="1">
+        <v>46174</v>
+      </c>
+      <c r="B199" t="s">
+        <v>396</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4129,6 +4146,7 @@
     <hyperlink r:id="rId193" ref="C196"/>
     <hyperlink r:id="rId194" ref="C197"/>
     <hyperlink r:id="rId195" ref="C198"/>
+    <hyperlink r:id="rId196" ref="C199"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: kth smallest element in a sorted matrix
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="400">
   <si>
     <t>date</t>
   </si>
@@ -1210,6 +1210,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/top-k-frequent-words/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kth smallest element in a sorted matrix</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/kth-smallest-element-in-a-sorted-matrix/</t>
   </si>
 </sst>
 </file>
@@ -3949,6 +3955,17 @@
         <v>397</v>
       </c>
     </row>
+    <row r="200" ht="14.25">
+      <c r="A200" s="1">
+        <v>46175</v>
+      </c>
+      <c r="B200" t="s">
+        <v>398</v>
+      </c>
+      <c r="C200" s="5" t="s">
+        <v>399</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4147,6 +4164,7 @@
     <hyperlink r:id="rId194" ref="C197"/>
     <hyperlink r:id="rId195" ref="C198"/>
     <hyperlink r:id="rId196" ref="C199"/>
+    <hyperlink r:id="rId197" ref="C200"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: cherry pickup II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="404">
   <si>
     <t>date</t>
   </si>
@@ -1222,6 +1222,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/k-closest-points-to-origin/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cherry pickup II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/cherry-pickup-ii/</t>
   </si>
 </sst>
 </file>
@@ -3983,6 +3989,17 @@
         <v>401</v>
       </c>
     </row>
+    <row r="202" ht="14.25">
+      <c r="A202" s="1">
+        <v>46177</v>
+      </c>
+      <c r="B202" t="s">
+        <v>402</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>403</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4183,6 +4200,7 @@
     <hyperlink r:id="rId196" ref="C199"/>
     <hyperlink r:id="rId197" ref="C200"/>
     <hyperlink r:id="rId198" ref="C201"/>
+    <hyperlink r:id="rId199" ref="C202"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: subset sum equal to k
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="408">
   <si>
     <t>date</t>
   </si>
@@ -1234,6 +1234,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/assign-cookies/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">subset sum problem</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/subset-sum-problem-1611555638/1</t>
   </si>
 </sst>
 </file>
@@ -4017,6 +4023,17 @@
         <v>405</v>
       </c>
     </row>
+    <row r="204" ht="14.25">
+      <c r="A204" s="1">
+        <v>46178</v>
+      </c>
+      <c r="B204" t="s">
+        <v>406</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4219,6 +4236,7 @@
     <hyperlink r:id="rId198" ref="C201"/>
     <hyperlink r:id="rId199" ref="C202"/>
     <hyperlink r:id="rId200" ref="C203"/>
+    <hyperlink r:id="rId201" ref="C204"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: partition equal subset sum
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="412">
   <si>
     <t>date</t>
   </si>
@@ -1246,6 +1246,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/reduce-array-size-to-the-half/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">partition equal subset sum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/partition-equal-subset-sum/</t>
   </si>
 </sst>
 </file>
@@ -4051,6 +4057,17 @@
         <v>409</v>
       </c>
     </row>
+    <row r="206" ht="14.25">
+      <c r="A206" s="1">
+        <v>46179</v>
+      </c>
+      <c r="B206" t="s">
+        <v>410</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>411</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4255,6 +4272,7 @@
     <hyperlink r:id="rId200" ref="C203"/>
     <hyperlink r:id="rId201" ref="C204"/>
     <hyperlink r:id="rId202" ref="C205"/>
+    <hyperlink r:id="rId203" ref="C206"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: min sum partition
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="416">
   <si>
     <t>date</t>
   </si>
@@ -1258,6 +1258,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/check-if-n-and-its-double-exist/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min. sum partition</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/minimum-sum-partition3317/1</t>
   </si>
 </sst>
 </file>
@@ -4085,6 +4091,17 @@
         <v>413</v>
       </c>
     </row>
+    <row r="208" ht="14.25">
+      <c r="A208" s="1">
+        <v>46180</v>
+      </c>
+      <c r="B208" t="s">
+        <v>414</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>415</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4291,6 +4308,7 @@
     <hyperlink r:id="rId202" ref="C205"/>
     <hyperlink r:id="rId203" ref="C206"/>
     <hyperlink r:id="rId204" ref="C207"/>
+    <hyperlink r:id="rId205" ref="C208"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: split a string in balanced string
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="418">
   <si>
     <t>date</t>
   </si>
@@ -1264,6 +1264,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/minimum-sum-partition3317/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">split a string in balanced strings</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/split-a-string-in-balanced-strings/</t>
   </si>
 </sst>
 </file>
@@ -4102,6 +4108,17 @@
         <v>415</v>
       </c>
     </row>
+    <row r="209" ht="14.25">
+      <c r="A209" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B209" t="s">
+        <v>416</v>
+      </c>
+      <c r="C209" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4309,6 +4326,7 @@
     <hyperlink r:id="rId203" ref="C206"/>
     <hyperlink r:id="rId204" ref="C207"/>
     <hyperlink r:id="rId205" ref="C208"/>
+    <hyperlink r:id="rId206" ref="C209"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: perfect sum problem
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="420">
   <si>
     <t>date</t>
   </si>
@@ -1270,6 +1270,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/split-a-string-in-balanced-strings/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">perfect sum problem</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/perfect-sum-problem5633/1</t>
   </si>
 </sst>
 </file>
@@ -4119,6 +4125,17 @@
         <v>417</v>
       </c>
     </row>
+    <row r="210" ht="14.25">
+      <c r="A210" s="1">
+        <v>46181</v>
+      </c>
+      <c r="B210" t="s">
+        <v>418</v>
+      </c>
+      <c r="C210" s="2" t="s">
+        <v>419</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4327,6 +4344,7 @@
     <hyperlink r:id="rId204" ref="C207"/>
     <hyperlink r:id="rId205" ref="C208"/>
     <hyperlink r:id="rId206" ref="C209"/>
+    <hyperlink r:id="rId207" ref="C210"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: min. cost to hire k workers
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="424">
   <si>
     <t>date</t>
   </si>
@@ -1282,6 +1282,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/partitions-with-given-difference/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">minimum cost to hire k workers</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-cost-to-hire-k-workers/</t>
   </si>
 </sst>
 </file>
@@ -4153,6 +4159,17 @@
         <v>421</v>
       </c>
     </row>
+    <row r="212" ht="14.25">
+      <c r="A212" s="1">
+        <v>46184</v>
+      </c>
+      <c r="B212" t="s">
+        <v>422</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>423</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -4363,6 +4380,7 @@
     <hyperlink r:id="rId206" ref="C209"/>
     <hyperlink r:id="rId207" ref="C210"/>
     <hyperlink r:id="rId208" ref="C211"/>
+    <hyperlink r:id="rId209" ref="C212"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: combination sum and rod cutting problem
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76CF44F-6E5B-41C3-BF84-6700073A4E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{011F183C-76B3-471B-8FB1-F3C9B8A318AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="436">
   <si>
     <t>date</t>
   </si>
@@ -1322,6 +1322,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/knapsack-with-duplicate-items4201/1</t>
+  </si>
+  <si>
+    <t>rod cutting problem</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/rod-cutting0840/1</t>
   </si>
 </sst>
 </file>
@@ -1592,7 +1598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D217"/>
+  <dimension ref="A1:D218"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -3978,6 +3984,17 @@
       </c>
       <c r="C217" s="4" t="s">
         <v>433</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A218" s="1">
+        <v>46188</v>
+      </c>
+      <c r="B218" t="s">
+        <v>434</v>
+      </c>
+      <c r="C218" s="4" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>
@@ -4196,8 +4213,9 @@
     <hyperlink ref="C215" r:id="rId212" xr:uid="{00000000-0004-0000-0000-0000D3000000}"/>
     <hyperlink ref="C216" r:id="rId213" xr:uid="{95DADF51-0029-47AE-8E17-84E67D521B48}"/>
     <hyperlink ref="C217" r:id="rId214" xr:uid="{B43A0CB5-E214-4BC9-8A56-6FD8D2AA8D99}"/>
+    <hyperlink ref="C218" r:id="rId215" xr:uid="{E551B356-82F4-4DEE-A9B6-4CAC836DBBCF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId215"/>
+  <pageSetup orientation="portrait" r:id="rId216"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: letter case permutation
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{011F183C-76B3-471B-8FB1-F3C9B8A318AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D76FD90-D778-49A7-A7AF-18EB26D67066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="438">
   <si>
     <t>date</t>
   </si>
@@ -1328,6 +1328,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/rod-cutting0840/1</t>
+  </si>
+  <si>
+    <t>letter case permutation</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/letter-case-permutation/</t>
   </si>
 </sst>
 </file>
@@ -1598,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D218"/>
+  <dimension ref="A1:D219"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -3995,6 +4001,17 @@
       </c>
       <c r="C218" s="4" t="s">
         <v>435</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A219" s="1">
+        <v>46189</v>
+      </c>
+      <c r="B219" t="s">
+        <v>436</v>
+      </c>
+      <c r="C219" s="4" t="s">
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -4214,8 +4231,9 @@
     <hyperlink ref="C216" r:id="rId213" xr:uid="{95DADF51-0029-47AE-8E17-84E67D521B48}"/>
     <hyperlink ref="C217" r:id="rId214" xr:uid="{B43A0CB5-E214-4BC9-8A56-6FD8D2AA8D99}"/>
     <hyperlink ref="C218" r:id="rId215" xr:uid="{E551B356-82F4-4DEE-A9B6-4CAC836DBBCF}"/>
+    <hyperlink ref="C219" r:id="rId216" xr:uid="{7A3C069D-6D65-4B6A-900E-33694EA1BBFA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId216"/>
+  <pageSetup orientation="portrait" r:id="rId217"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: restore IP addresses
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B67503-A513-4C7E-936E-D51959199C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F1D206-5A2B-4025-9DD3-110983A551CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="446">
   <si>
     <t>date</t>
   </si>
@@ -1352,6 +1352,12 @@
   </si>
   <si>
     <t>max. length of repeated subarray</t>
+  </si>
+  <si>
+    <t>restore ip addresses</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/restore-ip-addresses/</t>
   </si>
 </sst>
 </file>
@@ -1622,7 +1628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D222"/>
+  <dimension ref="A1:D223"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4063,6 +4069,17 @@
       </c>
       <c r="C222" s="4" t="s">
         <v>442</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A223" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B223" t="s">
+        <v>444</v>
+      </c>
+      <c r="C223" s="4" t="s">
+        <v>445</v>
       </c>
     </row>
   </sheetData>
@@ -4286,8 +4303,9 @@
     <hyperlink ref="C220" r:id="rId217" xr:uid="{2EA4DE40-0D59-4EAD-92A5-E1D46D0BEE9C}"/>
     <hyperlink ref="C221" r:id="rId218" xr:uid="{105DCDB4-957A-406A-9D90-380F57E707C1}"/>
     <hyperlink ref="C222" r:id="rId219" xr:uid="{76B8EA9C-8138-4EC3-9D55-58B047142A44}"/>
+    <hyperlink ref="C223" r:id="rId220" xr:uid="{599031F7-CBC5-47CC-8203-C2B0C0939432}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId220"/>
+  <pageSetup orientation="portrait" r:id="rId221"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: longest palindromic subsequnce
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F1D206-5A2B-4025-9DD3-110983A551CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5365E793-B11B-44B6-8EEC-25C656BAA46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="448">
   <si>
     <t>date</t>
   </si>
@@ -1358,6 +1358,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/restore-ip-addresses/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-palindromic-subsequence/</t>
+  </si>
+  <si>
+    <t>longest palindromic subsequence</t>
   </si>
 </sst>
 </file>
@@ -1628,11 +1634,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D224"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
-    <col min="2" max="2" width="51.36328125" bestFit="1"/>
+    <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="96.90625" bestFit="1"/>
     <col min="4" max="4" width="21.7265625" bestFit="1"/>
   </cols>
@@ -4080,6 +4086,17 @@
       </c>
       <c r="C223" s="4" t="s">
         <v>445</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A224" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B224" t="s">
+        <v>447</v>
+      </c>
+      <c r="C224" s="4" t="s">
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -4304,8 +4321,9 @@
     <hyperlink ref="C221" r:id="rId218" xr:uid="{105DCDB4-957A-406A-9D90-380F57E707C1}"/>
     <hyperlink ref="C222" r:id="rId219" xr:uid="{76B8EA9C-8138-4EC3-9D55-58B047142A44}"/>
     <hyperlink ref="C223" r:id="rId220" xr:uid="{599031F7-CBC5-47CC-8203-C2B0C0939432}"/>
+    <hyperlink ref="C224" r:id="rId221" xr:uid="{2520CA58-6164-40D0-A139-89878326E026}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId221"/>
+  <pageSetup orientation="portrait" r:id="rId222"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: combination sum III
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5365E793-B11B-44B6-8EEC-25C656BAA46D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FAEFE29-4E73-434A-B26C-2422C0A53D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="450">
   <si>
     <t>date</t>
   </si>
@@ -1364,6 +1364,12 @@
   </si>
   <si>
     <t>longest palindromic subsequence</t>
+  </si>
+  <si>
+    <t>combination sum III</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/combination-sum-iii</t>
   </si>
 </sst>
 </file>
@@ -1634,7 +1640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D224"/>
+  <dimension ref="A1:D225"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4097,6 +4103,17 @@
       </c>
       <c r="C224" s="4" t="s">
         <v>446</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A225" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B225" t="s">
+        <v>448</v>
+      </c>
+      <c r="C225" s="4" t="s">
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -4322,8 +4339,9 @@
     <hyperlink ref="C222" r:id="rId219" xr:uid="{76B8EA9C-8138-4EC3-9D55-58B047142A44}"/>
     <hyperlink ref="C223" r:id="rId220" xr:uid="{599031F7-CBC5-47CC-8203-C2B0C0939432}"/>
     <hyperlink ref="C224" r:id="rId221" xr:uid="{2520CA58-6164-40D0-A139-89878326E026}"/>
+    <hyperlink ref="C225" r:id="rId222" xr:uid="{74DCE01A-E90F-4335-BC09-6944BD888142}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId222"/>
+  <pageSetup orientation="portrait" r:id="rId223"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: min. deletion operations to make string s1 to s2
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAA13ED-2EDF-4050-909D-BAA292A9AF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B3610F-9C60-4BA7-A2E0-D5007AC27C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="456">
   <si>
     <t>date</t>
   </si>
@@ -1382,6 +1382,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/expression-add-operators/</t>
+  </si>
+  <si>
+    <t>Delete Operations For 2 strings</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/delete-operation-for-two-strings/</t>
   </si>
 </sst>
 </file>
@@ -1652,7 +1658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D227"/>
+  <dimension ref="A1:D228"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4148,6 +4154,17 @@
       </c>
       <c r="C227" s="4" t="s">
         <v>451</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A228" s="1">
+        <v>46192</v>
+      </c>
+      <c r="B228" t="s">
+        <v>454</v>
+      </c>
+      <c r="C228" s="4" t="s">
+        <v>455</v>
       </c>
     </row>
   </sheetData>
@@ -4376,8 +4393,9 @@
     <hyperlink ref="C225" r:id="rId222" xr:uid="{74DCE01A-E90F-4335-BC09-6944BD888142}"/>
     <hyperlink ref="C227" r:id="rId223" xr:uid="{F129DF05-12AE-4F8B-B901-10D9824B64C3}"/>
     <hyperlink ref="C226" r:id="rId224" xr:uid="{1738018E-5280-4EBF-B0E5-1880B2CBBC97}"/>
+    <hyperlink ref="C228" r:id="rId225" xr:uid="{6299FE99-DC4E-4BA9-A436-CA76F577B238}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId225"/>
+  <pageSetup orientation="portrait" r:id="rId226"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: find the highest altitude
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B3610F-9C60-4BA7-A2E0-D5007AC27C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4349746E-A776-4CD3-9D96-8C6B01DB3482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="458">
   <si>
     <t>date</t>
   </si>
@@ -1388,6 +1388,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/delete-operation-for-two-strings/</t>
+  </si>
+  <si>
+    <t>find the highest altitude</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-the-highest-altitude/</t>
   </si>
 </sst>
 </file>
@@ -1658,7 +1664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D228"/>
+  <dimension ref="A1:D229"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4165,6 +4171,17 @@
       </c>
       <c r="C228" s="4" t="s">
         <v>455</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A229" s="1">
+        <v>46192</v>
+      </c>
+      <c r="B229" t="s">
+        <v>456</v>
+      </c>
+      <c r="C229" s="4" t="s">
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -4394,8 +4411,9 @@
     <hyperlink ref="C227" r:id="rId223" xr:uid="{F129DF05-12AE-4F8B-B901-10D9824B64C3}"/>
     <hyperlink ref="C226" r:id="rId224" xr:uid="{1738018E-5280-4EBF-B0E5-1880B2CBBC97}"/>
     <hyperlink ref="C228" r:id="rId225" xr:uid="{6299FE99-DC4E-4BA9-A436-CA76F577B238}"/>
+    <hyperlink ref="C229" r:id="rId226" xr:uid="{CED6339E-BA64-40EC-809F-8F6683BD2FFB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId226"/>
+  <pageSetup orientation="portrait" r:id="rId227"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
problem: LIS using binary search
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8442EF1-A39D-40E3-B67C-6B67BB32E451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7057770A-0D13-45B9-8512-68BC4780DDA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="466">
   <si>
     <t>date</t>
   </si>
@@ -1412,6 +1412,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/wildcard-matching/</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/printing-longest-increasing-subsequence/1</t>
+  </si>
+  <si>
+    <t>printing LIS</t>
   </si>
 </sst>
 </file>
@@ -1682,7 +1688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D232"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4233,6 +4239,17 @@
       </c>
       <c r="C232" s="4" t="s">
         <v>463</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A233" s="1">
+        <v>46199</v>
+      </c>
+      <c r="B233" t="s">
+        <v>465</v>
+      </c>
+      <c r="C233" s="4" t="s">
+        <v>464</v>
       </c>
     </row>
   </sheetData>
@@ -4466,8 +4483,9 @@
     <hyperlink ref="C230" r:id="rId227" xr:uid="{18B3952D-D773-4220-83A8-5DFCBE47BE6B}"/>
     <hyperlink ref="C231" r:id="rId228" xr:uid="{B5E70D10-CDC3-4746-8E93-23E7DE722147}"/>
     <hyperlink ref="C232" r:id="rId229" xr:uid="{7874E577-FFBF-45D8-811A-8A6780B02C8C}"/>
+    <hyperlink ref="C233" r:id="rId230" xr:uid="{1AB23B31-A231-42A7-92AD-E1E7D40A5E67}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId230"/>
+  <pageSetup orientation="portrait" r:id="rId231"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: longest string chain
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E991288-1FC5-48D7-8DBF-5BBFFA897A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6137FAF8-6CAC-4224-B628-0B8BB076EB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="470">
   <si>
     <t>date</t>
   </si>
@@ -1424,6 +1424,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/largest-divisible-subset/</t>
+  </si>
+  <si>
+    <t>longest string chain</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-string-chain/</t>
   </si>
 </sst>
 </file>
@@ -1694,7 +1700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D234"/>
+  <dimension ref="A1:D235"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4267,6 +4273,17 @@
       </c>
       <c r="C234" s="4" t="s">
         <v>467</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A235" s="1">
+        <v>46201</v>
+      </c>
+      <c r="B235" t="s">
+        <v>468</v>
+      </c>
+      <c r="C235" s="4" t="s">
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -4502,8 +4519,9 @@
     <hyperlink ref="C232" r:id="rId229" xr:uid="{7874E577-FFBF-45D8-811A-8A6780B02C8C}"/>
     <hyperlink ref="C233" r:id="rId230" xr:uid="{1AB23B31-A231-42A7-92AD-E1E7D40A5E67}"/>
     <hyperlink ref="C234" r:id="rId231" xr:uid="{D41A7E5E-D532-4BBD-9F17-A2984DAE138E}"/>
+    <hyperlink ref="C235" r:id="rId232" xr:uid="{B10F0A9A-6F8C-4054-8A2E-B815C6782EAE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId232"/>
+  <pageSetup orientation="portrait" r:id="rId233"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: infix to postfix
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6137FAF8-6CAC-4224-B628-0B8BB076EB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F5CDFB-DEB2-4D0F-9335-70E2556BA730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="472">
   <si>
     <t>date</t>
   </si>
@@ -1430,6 +1430,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/longest-string-chain/</t>
+  </si>
+  <si>
+    <t>infix to postfix</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/infix-to-postfix-1587115620/1</t>
   </si>
 </sst>
 </file>
@@ -1700,7 +1706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D235"/>
+  <dimension ref="A1:D236"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4284,6 +4290,17 @@
       </c>
       <c r="C235" s="4" t="s">
         <v>469</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A236" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B236" t="s">
+        <v>470</v>
+      </c>
+      <c r="C236" s="4" t="s">
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -4520,8 +4537,9 @@
     <hyperlink ref="C233" r:id="rId230" xr:uid="{1AB23B31-A231-42A7-92AD-E1E7D40A5E67}"/>
     <hyperlink ref="C234" r:id="rId231" xr:uid="{D41A7E5E-D532-4BBD-9F17-A2984DAE138E}"/>
     <hyperlink ref="C235" r:id="rId232" xr:uid="{B10F0A9A-6F8C-4054-8A2E-B815C6782EAE}"/>
+    <hyperlink ref="C236" r:id="rId233" xr:uid="{38790754-C274-4AF5-BD96-395819B5E1D6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId233"/>
+  <pageSetup orientation="portrait" r:id="rId234"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: infix to prefix
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F5CDFB-DEB2-4D0F-9335-70E2556BA730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C36C77A-D36A-4D16-8B58-BC23C39C0EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="474">
   <si>
     <t>date</t>
   </si>
@@ -1436,6 +1436,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/infix-to-postfix-1587115620/1</t>
+  </si>
+  <si>
+    <t>infix to prefix</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/infix-to-prefix-notation/1</t>
   </si>
 </sst>
 </file>
@@ -1706,7 +1712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D236"/>
+  <dimension ref="A1:D237"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4301,6 +4307,17 @@
       </c>
       <c r="C236" s="4" t="s">
         <v>471</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A237" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B237" t="s">
+        <v>472</v>
+      </c>
+      <c r="C237" s="4" t="s">
+        <v>473</v>
       </c>
     </row>
   </sheetData>
@@ -4538,8 +4555,9 @@
     <hyperlink ref="C234" r:id="rId231" xr:uid="{D41A7E5E-D532-4BBD-9F17-A2984DAE138E}"/>
     <hyperlink ref="C235" r:id="rId232" xr:uid="{B10F0A9A-6F8C-4054-8A2E-B815C6782EAE}"/>
     <hyperlink ref="C236" r:id="rId233" xr:uid="{38790754-C274-4AF5-BD96-395819B5E1D6}"/>
+    <hyperlink ref="C237" r:id="rId234" xr:uid="{A4ED1F23-DC17-4631-9B96-1A63EBD6DE41}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId234"/>
+  <pageSetup orientation="portrait" r:id="rId235"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problems: all conversion combos of prefix, infix, postfix
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C36C77A-D36A-4D16-8B58-BC23C39C0EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225A74C6-9486-4BBF-8507-231CDEB1DDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="482">
   <si>
     <t>date</t>
   </si>
@@ -1442,6 +1442,30 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/infix-to-prefix-notation/1</t>
+  </si>
+  <si>
+    <t>prefix to infix</t>
+  </si>
+  <si>
+    <t>prefix to postfix</t>
+  </si>
+  <si>
+    <t>postfix to infix</t>
+  </si>
+  <si>
+    <t>postfix to prefix</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/prefix-to-postfix-conversion/1</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/prefix-to-infix-conversion/1</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/postfix-to-infix-conversion/1</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/postfix-to-prefix-conversion/1</t>
   </si>
 </sst>
 </file>
@@ -1712,7 +1736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D237"/>
+  <dimension ref="A1:D241"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4318,6 +4342,50 @@
       </c>
       <c r="C237" s="4" t="s">
         <v>473</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A238" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B238" t="s">
+        <v>474</v>
+      </c>
+      <c r="C238" s="4" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A239" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B239" t="s">
+        <v>475</v>
+      </c>
+      <c r="C239" s="4" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A240" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B240" t="s">
+        <v>476</v>
+      </c>
+      <c r="C240" s="4" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A241" s="1">
+        <v>46205</v>
+      </c>
+      <c r="B241" t="s">
+        <v>477</v>
+      </c>
+      <c r="C241" s="4" t="s">
+        <v>481</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Problem: Next Greater Element leetcode
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225A74C6-9486-4BBF-8507-231CDEB1DDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C31794-6374-41F9-93F7-DEF1946F8CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="484">
   <si>
     <t>date</t>
   </si>
@@ -1466,6 +1466,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/postfix-to-prefix-conversion/1</t>
+  </si>
+  <si>
+    <t>Next Greater Element(Leetcode 496)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/next-greater-element-i/</t>
   </si>
 </sst>
 </file>
@@ -1736,7 +1742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D241"/>
+  <dimension ref="A1:D242"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4386,6 +4392,17 @@
       </c>
       <c r="C241" s="4" t="s">
         <v>481</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A242" s="1">
+        <v>46206</v>
+      </c>
+      <c r="B242" t="s">
+        <v>482</v>
+      </c>
+      <c r="C242" s="4" t="s">
+        <v>483</v>
       </c>
     </row>
   </sheetData>
@@ -4624,8 +4641,9 @@
     <hyperlink ref="C235" r:id="rId232" xr:uid="{B10F0A9A-6F8C-4054-8A2E-B815C6782EAE}"/>
     <hyperlink ref="C236" r:id="rId233" xr:uid="{38790754-C274-4AF5-BD96-395819B5E1D6}"/>
     <hyperlink ref="C237" r:id="rId234" xr:uid="{A4ED1F23-DC17-4631-9B96-1A63EBD6DE41}"/>
+    <hyperlink ref="C242" r:id="rId235" xr:uid="{DD2956C1-6E6D-4BD7-B2F5-DDD903E3E7E5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId235"/>
+  <pageSetup orientation="portrait" r:id="rId236"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: count no. of NGEs in the right
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C31794-6374-41F9-93F7-DEF1946F8CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BA4685-A3C6-40A8-B263-BB14A1E22BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="486">
   <si>
     <t>date</t>
   </si>
@@ -1472,6 +1472,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/next-greater-element-i/</t>
+  </si>
+  <si>
+    <t>Number of nges to the Right</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/number-of-nges-to-the-right/1</t>
   </si>
 </sst>
 </file>
@@ -1742,7 +1748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D242"/>
+  <dimension ref="A1:D243"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4403,6 +4409,17 @@
       </c>
       <c r="C242" s="4" t="s">
         <v>483</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A243" s="1">
+        <v>46207</v>
+      </c>
+      <c r="B243" t="s">
+        <v>484</v>
+      </c>
+      <c r="C243" s="4" t="s">
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -4642,8 +4659,9 @@
     <hyperlink ref="C236" r:id="rId233" xr:uid="{38790754-C274-4AF5-BD96-395819B5E1D6}"/>
     <hyperlink ref="C237" r:id="rId234" xr:uid="{A4ED1F23-DC17-4631-9B96-1A63EBD6DE41}"/>
     <hyperlink ref="C242" r:id="rId235" xr:uid="{DD2956C1-6E6D-4BD7-B2F5-DDD903E3E7E5}"/>
+    <hyperlink ref="C243" r:id="rId236" xr:uid="{5108CAD3-9717-409E-81C3-3C733511C655}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId236"/>
+  <pageSetup orientation="portrait" r:id="rId237"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: sum of subarray minimums
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1BA4685-A3C6-40A8-B263-BB14A1E22BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969E3F79-A415-411A-91D6-4D9B9FC49FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="488">
   <si>
     <t>date</t>
   </si>
@@ -1478,6 +1478,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/number-of-nges-to-the-right/1</t>
+  </si>
+  <si>
+    <t>sum of subarray minimum</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sum-of-subarray-minimums/</t>
   </si>
 </sst>
 </file>
@@ -1748,7 +1754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D243"/>
+  <dimension ref="A1:D244"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4420,6 +4426,17 @@
       </c>
       <c r="C243" s="4" t="s">
         <v>485</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A244" s="1">
+        <v>46208</v>
+      </c>
+      <c r="B244" t="s">
+        <v>486</v>
+      </c>
+      <c r="C244" s="4" t="s">
+        <v>487</v>
       </c>
     </row>
   </sheetData>
@@ -4660,8 +4677,9 @@
     <hyperlink ref="C237" r:id="rId234" xr:uid="{A4ED1F23-DC17-4631-9B96-1A63EBD6DE41}"/>
     <hyperlink ref="C242" r:id="rId235" xr:uid="{DD2956C1-6E6D-4BD7-B2F5-DDD903E3E7E5}"/>
     <hyperlink ref="C243" r:id="rId236" xr:uid="{5108CAD3-9717-409E-81C3-3C733511C655}"/>
+    <hyperlink ref="C244" r:id="rId237" xr:uid="{235C0F52-84F8-4BE3-A2C8-5D7907A2C49D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId237"/>
+  <pageSetup orientation="portrait" r:id="rId238"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: valid paranthesis string
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969E3F79-A415-411A-91D6-4D9B9FC49FB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE91A19-263C-4476-8859-1938DA2AC820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="490">
   <si>
     <t>date</t>
   </si>
@@ -1484,6 +1484,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/sum-of-subarray-minimums/</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/valid-parenthesis-string/</t>
+  </si>
+  <si>
+    <t>valid parenthesis string</t>
   </si>
 </sst>
 </file>
@@ -1754,7 +1760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D244"/>
+  <dimension ref="A1:D245"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4437,6 +4443,17 @@
       </c>
       <c r="C244" s="4" t="s">
         <v>487</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A245" s="1">
+        <v>46208</v>
+      </c>
+      <c r="B245" t="s">
+        <v>489</v>
+      </c>
+      <c r="C245" s="4" t="s">
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -4678,8 +4695,9 @@
     <hyperlink ref="C242" r:id="rId235" xr:uid="{DD2956C1-6E6D-4BD7-B2F5-DDD903E3E7E5}"/>
     <hyperlink ref="C243" r:id="rId236" xr:uid="{5108CAD3-9717-409E-81C3-3C733511C655}"/>
     <hyperlink ref="C244" r:id="rId237" xr:uid="{235C0F52-84F8-4BE3-A2C8-5D7907A2C49D}"/>
+    <hyperlink ref="C245" r:id="rId238" xr:uid="{DFF0B69B-C0EA-400B-917C-0EC5DFF1FD6D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId238"/>
+  <pageSetup orientation="portrait" r:id="rId239"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: min. insertions to balance paranthesis
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE91A19-263C-4476-8859-1938DA2AC820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{972D8412-5A0E-45EE-A853-D05F6EB5AFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="492">
   <si>
     <t>date</t>
   </si>
@@ -1490,6 +1490,12 @@
   </si>
   <si>
     <t>valid parenthesis string</t>
+  </si>
+  <si>
+    <t>min. insertions to balance a paranthesis string</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-insertions-to-balance-a-parentheses-string/</t>
   </si>
 </sst>
 </file>
@@ -1760,7 +1766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D245"/>
+  <dimension ref="A1:D246"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4454,6 +4460,17 @@
       </c>
       <c r="C245" s="4" t="s">
         <v>488</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A246" s="1">
+        <v>46208</v>
+      </c>
+      <c r="B246" t="s">
+        <v>490</v>
+      </c>
+      <c r="C246" s="4" t="s">
+        <v>491</v>
       </c>
     </row>
   </sheetData>
@@ -4696,8 +4713,9 @@
     <hyperlink ref="C243" r:id="rId236" xr:uid="{5108CAD3-9717-409E-81C3-3C733511C655}"/>
     <hyperlink ref="C244" r:id="rId237" xr:uid="{235C0F52-84F8-4BE3-A2C8-5D7907A2C49D}"/>
     <hyperlink ref="C245" r:id="rId238" xr:uid="{DFF0B69B-C0EA-400B-917C-0EC5DFF1FD6D}"/>
+    <hyperlink ref="C246" r:id="rId239" xr:uid="{9023AC70-E3A5-4F67-B06B-E94BE5991317}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId239"/>
+  <pageSetup orientation="portrait" r:id="rId240"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: DSU and Kruskals Algo
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0327DAE8-B3B7-40BD-9B4F-A4CF1E9A5F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EF8FFA-9AB0-41AE-82B3-14F60E9F66B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="498">
   <si>
     <t>date</t>
   </si>
@@ -1508,6 +1508,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/disjoint-set-union-find/1</t>
+  </si>
+  <si>
+    <t>Kruskal's Algorithm</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/minimum-spanning-tree-kruskals-algorithm/1</t>
   </si>
 </sst>
 </file>
@@ -1778,7 +1784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D248"/>
+  <dimension ref="A1:D249"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4505,6 +4511,17 @@
       </c>
       <c r="C248" s="4" t="s">
         <v>495</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A249" s="1">
+        <v>46209</v>
+      </c>
+      <c r="B249" t="s">
+        <v>496</v>
+      </c>
+      <c r="C249" s="4" t="s">
+        <v>497</v>
       </c>
     </row>
   </sheetData>
@@ -4750,8 +4767,9 @@
     <hyperlink ref="C246" r:id="rId239" xr:uid="{9023AC70-E3A5-4F67-B06B-E94BE5991317}"/>
     <hyperlink ref="C247" r:id="rId240" xr:uid="{1713DF23-F8AC-45D8-B30B-58E80AA38080}"/>
     <hyperlink ref="C248" r:id="rId241" xr:uid="{197C6370-568D-44C0-BEAE-AECCDC36B606}"/>
+    <hyperlink ref="C249" r:id="rId242" xr:uid="{8C008180-707B-42C1-9BBD-1CD49C8072B0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId242"/>
+  <pageSetup orientation="portrait" r:id="rId243"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: sum of subarray ranges
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0595E6C6-B485-43E6-B8E1-C03F8C959FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB47E27-84A6-4CE8-A84E-361BFCB05F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="502">
   <si>
     <t>date</t>
   </si>
@@ -1520,6 +1520,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/minimum-spanning-tree/1</t>
+  </si>
+  <si>
+    <t>sum of subarray ranges</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sum-of-subarray-ranges/</t>
   </si>
 </sst>
 </file>
@@ -1790,7 +1796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D250"/>
+  <dimension ref="A1:D251"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4539,6 +4545,17 @@
       </c>
       <c r="C250" s="4" t="s">
         <v>499</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A251" s="1">
+        <v>46210</v>
+      </c>
+      <c r="B251" t="s">
+        <v>500</v>
+      </c>
+      <c r="C251" s="4" t="s">
+        <v>501</v>
       </c>
     </row>
   </sheetData>
@@ -4786,8 +4803,9 @@
     <hyperlink ref="C248" r:id="rId241" xr:uid="{197C6370-568D-44C0-BEAE-AECCDC36B606}"/>
     <hyperlink ref="C249" r:id="rId242" xr:uid="{8C008180-707B-42C1-9BBD-1CD49C8072B0}"/>
     <hyperlink ref="C250" r:id="rId243" xr:uid="{F669F69C-E86B-462F-A826-A607851D501A}"/>
+    <hyperlink ref="C251" r:id="rId244" xr:uid="{D5A8508A-1973-4591-89E7-CCAD28B46C0A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId244"/>
+  <pageSetup orientation="portrait" r:id="rId245"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Floyd Warshall Algo
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB47E27-84A6-4CE8-A84E-361BFCB05F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54B7B8E-9CB3-428D-903A-7426EEED1A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="504">
   <si>
     <t>date</t>
   </si>
@@ -1526,6 +1526,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/sum-of-subarray-ranges/</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/implementing-floyd-warshall2042/1</t>
+  </si>
+  <si>
+    <t>floyd warshall algo</t>
   </si>
 </sst>
 </file>
@@ -1796,7 +1802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D251"/>
+  <dimension ref="A1:D252"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4556,6 +4562,17 @@
       </c>
       <c r="C251" s="4" t="s">
         <v>501</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A252" s="1">
+        <v>46210</v>
+      </c>
+      <c r="B252" t="s">
+        <v>503</v>
+      </c>
+      <c r="C252" s="4" t="s">
+        <v>502</v>
       </c>
     </row>
   </sheetData>
@@ -4804,8 +4821,9 @@
     <hyperlink ref="C249" r:id="rId242" xr:uid="{8C008180-707B-42C1-9BBD-1CD49C8072B0}"/>
     <hyperlink ref="C250" r:id="rId243" xr:uid="{F669F69C-E86B-462F-A826-A607851D501A}"/>
     <hyperlink ref="C251" r:id="rId244" xr:uid="{D5A8508A-1973-4591-89E7-CCAD28B46C0A}"/>
+    <hyperlink ref="C252" r:id="rId245" xr:uid="{016203F2-EB56-4982-A892-25DD108086A8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId245"/>
+  <pageSetup orientation="portrait" r:id="rId246"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: remove k digits
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54B7B8E-9CB3-428D-903A-7426EEED1A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2071635-41FF-489F-985E-3557BA572441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="506">
   <si>
     <t>date</t>
   </si>
@@ -1532,6 +1532,12 @@
   </si>
   <si>
     <t>floyd warshall algo</t>
+  </si>
+  <si>
+    <t>remove k digits</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-k-digits/</t>
   </si>
 </sst>
 </file>
@@ -1802,7 +1808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D252"/>
+  <dimension ref="A1:D253"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4573,6 +4579,17 @@
       </c>
       <c r="C252" s="4" t="s">
         <v>502</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A253" s="1">
+        <v>46211</v>
+      </c>
+      <c r="B253" t="s">
+        <v>504</v>
+      </c>
+      <c r="C253" s="4" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -4822,8 +4839,9 @@
     <hyperlink ref="C250" r:id="rId243" xr:uid="{F669F69C-E86B-462F-A826-A607851D501A}"/>
     <hyperlink ref="C251" r:id="rId244" xr:uid="{D5A8508A-1973-4591-89E7-CCAD28B46C0A}"/>
     <hyperlink ref="C252" r:id="rId245" xr:uid="{016203F2-EB56-4982-A892-25DD108086A8}"/>
+    <hyperlink ref="C253" r:id="rId246" xr:uid="{111A54C6-EC42-4204-8955-EB1EA3274B9E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId246"/>
+  <pageSetup orientation="portrait" r:id="rId247"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problems: sliding window maximum, online stock span and celebrity problem
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2071635-41FF-489F-985E-3557BA572441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5108D2C-D387-4B4A-B16B-F59E558F3EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="508">
   <si>
     <t>date</t>
   </si>
@@ -1538,6 +1538,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-k-digits/</t>
+  </si>
+  <si>
+    <t>the celebrity problem</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/the-celebrity-problem/1</t>
   </si>
 </sst>
 </file>
@@ -1808,7 +1814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D253"/>
+  <dimension ref="A1:D254"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4590,6 +4596,17 @@
       </c>
       <c r="C253" s="4" t="s">
         <v>505</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A254" s="1">
+        <v>46214</v>
+      </c>
+      <c r="B254" t="s">
+        <v>506</v>
+      </c>
+      <c r="C254" s="4" t="s">
+        <v>507</v>
       </c>
     </row>
   </sheetData>
@@ -4840,8 +4857,9 @@
     <hyperlink ref="C251" r:id="rId244" xr:uid="{D5A8508A-1973-4591-89E7-CCAD28B46C0A}"/>
     <hyperlink ref="C252" r:id="rId245" xr:uid="{016203F2-EB56-4982-A892-25DD108086A8}"/>
     <hyperlink ref="C253" r:id="rId246" xr:uid="{111A54C6-EC42-4204-8955-EB1EA3274B9E}"/>
+    <hyperlink ref="C254" r:id="rId247" xr:uid="{DA7F8667-832E-4D96-A725-FAE3103D7CF4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId247"/>
+  <pageSetup orientation="portrait" r:id="rId248"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: LRU Cache and LFU Cache
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5108D2C-D387-4B4A-B16B-F59E558F3EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D802D938-5236-43DA-82AD-DD952D0AD75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="510">
   <si>
     <t>date</t>
   </si>
@@ -1544,6 +1544,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/the-celebrity-problem/1</t>
+  </si>
+  <si>
+    <t>LFU Cache</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/lfu-cache/</t>
   </si>
 </sst>
 </file>
@@ -1814,7 +1820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D254"/>
+  <dimension ref="A1:D255"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4607,6 +4613,17 @@
       </c>
       <c r="C254" s="4" t="s">
         <v>507</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A255" s="1">
+        <v>46215</v>
+      </c>
+      <c r="B255" t="s">
+        <v>508</v>
+      </c>
+      <c r="C255" s="4" t="s">
+        <v>509</v>
       </c>
     </row>
   </sheetData>
@@ -4858,8 +4875,9 @@
     <hyperlink ref="C252" r:id="rId245" xr:uid="{016203F2-EB56-4982-A892-25DD108086A8}"/>
     <hyperlink ref="C253" r:id="rId246" xr:uid="{111A54C6-EC42-4204-8955-EB1EA3274B9E}"/>
     <hyperlink ref="C254" r:id="rId247" xr:uid="{DA7F8667-832E-4D96-A725-FAE3103D7CF4}"/>
+    <hyperlink ref="C255" r:id="rId248" xr:uid="{630B899E-C2BF-4EC7-B738-085C119D0E9B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId248"/>
+  <pageSetup orientation="portrait" r:id="rId249"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem : insertion and deletion in Linked List
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D802D938-5236-43DA-82AD-DD952D0AD75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480FBD1F-BD33-4866-9A3A-8E67D2429657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="512">
   <si>
     <t>date</t>
   </si>
@@ -1550,6 +1550,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/lfu-cache/</t>
+  </si>
+  <si>
+    <t>delete nodes in a linked list</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/delete-node-in-a-linked-list/</t>
   </si>
 </sst>
 </file>
@@ -1820,7 +1826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D255"/>
+  <dimension ref="A1:D256"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4624,6 +4630,17 @@
       </c>
       <c r="C255" s="4" t="s">
         <v>509</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A256" s="1">
+        <v>46216</v>
+      </c>
+      <c r="B256" t="s">
+        <v>510</v>
+      </c>
+      <c r="C256" s="4" t="s">
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -4876,8 +4893,9 @@
     <hyperlink ref="C253" r:id="rId246" xr:uid="{111A54C6-EC42-4204-8955-EB1EA3274B9E}"/>
     <hyperlink ref="C254" r:id="rId247" xr:uid="{DA7F8667-832E-4D96-A725-FAE3103D7CF4}"/>
     <hyperlink ref="C255" r:id="rId248" xr:uid="{630B899E-C2BF-4EC7-B738-085C119D0E9B}"/>
+    <hyperlink ref="C256" r:id="rId249" xr:uid="{22C2D33A-FCE9-4E27-A877-0C6C9C2B657C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId249"/>
+  <pageSetup orientation="portrait" r:id="rId250"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: delete kth position of doubly linked list
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480FBD1F-BD33-4866-9A3A-8E67D2429657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0825B938-3E21-49C5-80BF-89351B412C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="514">
   <si>
     <t>date</t>
   </si>
@@ -1556,6 +1556,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/delete-node-in-a-linked-list/</t>
+  </si>
+  <si>
+    <t>delete kth node in a doubly linked list</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/delete-node-in-doubly-linked-list/1</t>
   </si>
 </sst>
 </file>
@@ -1826,7 +1832,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D256"/>
+  <dimension ref="A1:D257"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4641,6 +4647,17 @@
       </c>
       <c r="C256" s="4" t="s">
         <v>511</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A257" s="1">
+        <v>46216</v>
+      </c>
+      <c r="B257" t="s">
+        <v>512</v>
+      </c>
+      <c r="C257" s="4" t="s">
+        <v>513</v>
       </c>
     </row>
   </sheetData>
@@ -4894,8 +4911,9 @@
     <hyperlink ref="C254" r:id="rId247" xr:uid="{DA7F8667-832E-4D96-A725-FAE3103D7CF4}"/>
     <hyperlink ref="C255" r:id="rId248" xr:uid="{630B899E-C2BF-4EC7-B738-085C119D0E9B}"/>
     <hyperlink ref="C256" r:id="rId249" xr:uid="{22C2D33A-FCE9-4E27-A877-0C6C9C2B657C}"/>
+    <hyperlink ref="C257" r:id="rId250" xr:uid="{CF96F2CE-2B3C-41A1-8AC2-ECEB22D62DE5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId250"/>
+  <pageSetup orientation="portrait" r:id="rId251"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: reverse a doubly linked list
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0825B938-3E21-49C5-80BF-89351B412C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F7160C-05D3-45FF-811E-83FEADA85EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="516">
   <si>
     <t>date</t>
   </si>
@@ -1562,6 +1562,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/delete-node-in-doubly-linked-list/1</t>
+  </si>
+  <si>
+    <t>reverse a doubly linked list</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/reverse-a-doubly-linked-list/1</t>
   </si>
 </sst>
 </file>
@@ -1832,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D257"/>
+  <dimension ref="A1:D258"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4658,6 +4664,17 @@
       </c>
       <c r="C257" s="4" t="s">
         <v>513</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A258" s="1">
+        <v>46216</v>
+      </c>
+      <c r="B258" t="s">
+        <v>514</v>
+      </c>
+      <c r="C258" s="4" t="s">
+        <v>515</v>
       </c>
     </row>
   </sheetData>
@@ -4912,8 +4929,9 @@
     <hyperlink ref="C255" r:id="rId248" xr:uid="{630B899E-C2BF-4EC7-B738-085C119D0E9B}"/>
     <hyperlink ref="C256" r:id="rId249" xr:uid="{22C2D33A-FCE9-4E27-A877-0C6C9C2B657C}"/>
     <hyperlink ref="C257" r:id="rId250" xr:uid="{CF96F2CE-2B3C-41A1-8AC2-ECEB22D62DE5}"/>
+    <hyperlink ref="C258" r:id="rId251" xr:uid="{01CAD5D8-2CBC-4B4E-A655-ED64B12D54F8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId251"/>
+  <pageSetup orientation="portrait" r:id="rId252"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: find middle node of Linked List
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F7160C-05D3-45FF-811E-83FEADA85EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD17F96-4B97-4112-86FF-248F49EACF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="518">
   <si>
     <t>date</t>
   </si>
@@ -1568,6 +1568,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/reverse-a-doubly-linked-list/1</t>
+  </si>
+  <si>
+    <t>find middle node of Linked List</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
   </si>
 </sst>
 </file>
@@ -1838,7 +1844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D258"/>
+  <dimension ref="A1:D259"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4675,6 +4681,17 @@
       </c>
       <c r="C258" s="4" t="s">
         <v>515</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A259" s="1">
+        <v>46217</v>
+      </c>
+      <c r="B259" t="s">
+        <v>516</v>
+      </c>
+      <c r="C259" s="4" t="s">
+        <v>517</v>
       </c>
     </row>
   </sheetData>
@@ -4930,8 +4947,9 @@
     <hyperlink ref="C256" r:id="rId249" xr:uid="{22C2D33A-FCE9-4E27-A877-0C6C9C2B657C}"/>
     <hyperlink ref="C257" r:id="rId250" xr:uid="{CF96F2CE-2B3C-41A1-8AC2-ECEB22D62DE5}"/>
     <hyperlink ref="C258" r:id="rId251" xr:uid="{01CAD5D8-2CBC-4B4E-A655-ED64B12D54F8}"/>
+    <hyperlink ref="C259" r:id="rId252" xr:uid="{3A0E5455-0676-4565-AD44-6E6DF0129B1C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId252"/>
+  <pageSetup orientation="portrait" r:id="rId253"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: reverse a linked list
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD17F96-4B97-4112-86FF-248F49EACF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75057E72-A634-45E6-A370-96C34CE435DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="520">
   <si>
     <t>date</t>
   </si>
@@ -1574,6 +1574,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/middle-of-the-linked-list/</t>
+  </si>
+  <si>
+    <t>reverse a linked list</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-linked-list/</t>
   </si>
 </sst>
 </file>
@@ -1844,7 +1850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D259"/>
+  <dimension ref="A1:D260"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4692,6 +4698,17 @@
       </c>
       <c r="C259" s="4" t="s">
         <v>517</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A260" s="1">
+        <v>46217</v>
+      </c>
+      <c r="B260" t="s">
+        <v>518</v>
+      </c>
+      <c r="C260" s="4" t="s">
+        <v>519</v>
       </c>
     </row>
   </sheetData>
@@ -4948,8 +4965,9 @@
     <hyperlink ref="C257" r:id="rId250" xr:uid="{CF96F2CE-2B3C-41A1-8AC2-ECEB22D62DE5}"/>
     <hyperlink ref="C258" r:id="rId251" xr:uid="{01CAD5D8-2CBC-4B4E-A655-ED64B12D54F8}"/>
     <hyperlink ref="C259" r:id="rId252" xr:uid="{3A0E5455-0676-4565-AD44-6E6DF0129B1C}"/>
+    <hyperlink ref="C260" r:id="rId253" xr:uid="{CBB4B852-B427-4290-B862-B694BFFF78A1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId253"/>
+  <pageSetup orientation="portrait" r:id="rId254"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Hard DP Problem
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75057E72-A634-45E6-A370-96C34CE435DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B19775E-F310-4E16-8683-A4093E738C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="522">
   <si>
     <t>date</t>
   </si>
@@ -1580,6 +1580,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/reverse-linked-list/</t>
+  </si>
+  <si>
+    <t>min. steps to convert string with operations</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-steps-to-convert-string-with-operations/</t>
   </si>
 </sst>
 </file>
@@ -1850,7 +1856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D260"/>
+  <dimension ref="A1:D261"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4709,6 +4715,17 @@
       </c>
       <c r="C260" s="4" t="s">
         <v>519</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A261" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B261" t="s">
+        <v>520</v>
+      </c>
+      <c r="C261" s="4" t="s">
+        <v>521</v>
       </c>
     </row>
   </sheetData>
@@ -4966,8 +4983,9 @@
     <hyperlink ref="C258" r:id="rId251" xr:uid="{01CAD5D8-2CBC-4B4E-A655-ED64B12D54F8}"/>
     <hyperlink ref="C259" r:id="rId252" xr:uid="{3A0E5455-0676-4565-AD44-6E6DF0129B1C}"/>
     <hyperlink ref="C260" r:id="rId253" xr:uid="{CBB4B852-B427-4290-B862-B694BFFF78A1}"/>
+    <hyperlink ref="C261" r:id="rId254" xr:uid="{8380DBBE-C42A-44E0-A990-3F6D492608A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId254"/>
+  <pageSetup orientation="portrait" r:id="rId255"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: LL cycle II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B19775E-F310-4E16-8683-A4093E738C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B5E1A9-349A-4981-9F1E-692F3410483B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="524">
   <si>
     <t>date</t>
   </si>
@@ -1586,6 +1586,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-steps-to-convert-string-with-operations/</t>
+  </si>
+  <si>
+    <t>Linked List Cycle II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/linked-list-cycle-ii/</t>
   </si>
 </sst>
 </file>
@@ -1856,7 +1862,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D261"/>
+  <dimension ref="A1:D262"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4726,6 +4732,17 @@
       </c>
       <c r="C261" s="4" t="s">
         <v>521</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A262" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B262" t="s">
+        <v>522</v>
+      </c>
+      <c r="C262" s="4" t="s">
+        <v>523</v>
       </c>
     </row>
   </sheetData>
@@ -4984,8 +5001,9 @@
     <hyperlink ref="C259" r:id="rId252" xr:uid="{3A0E5455-0676-4565-AD44-6E6DF0129B1C}"/>
     <hyperlink ref="C260" r:id="rId253" xr:uid="{CBB4B852-B427-4290-B862-B694BFFF78A1}"/>
     <hyperlink ref="C261" r:id="rId254" xr:uid="{8380DBBE-C42A-44E0-A990-3F6D492608A5}"/>
+    <hyperlink ref="C262" r:id="rId255" xr:uid="{92C39D19-1599-44F9-8163-8F5DDB6B030A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId255"/>
+  <pageSetup orientation="portrait" r:id="rId256"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: Length of loop in LL
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B5E1A9-349A-4981-9F1E-692F3410483B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB414A5C-E654-4F5F-B1AE-7868954A1DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="526">
   <si>
     <t>date</t>
   </si>
@@ -1592,6 +1592,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/linked-list-cycle-ii/</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/find-length-of-loop/1</t>
+  </si>
+  <si>
+    <t>find length of loop in Linked List</t>
   </si>
 </sst>
 </file>
@@ -1862,7 +1868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D262"/>
+  <dimension ref="A1:D263"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4743,6 +4749,17 @@
       </c>
       <c r="C262" s="4" t="s">
         <v>523</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A263" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B263" t="s">
+        <v>525</v>
+      </c>
+      <c r="C263" s="4" t="s">
+        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -5002,8 +5019,9 @@
     <hyperlink ref="C260" r:id="rId253" xr:uid="{CBB4B852-B427-4290-B862-B694BFFF78A1}"/>
     <hyperlink ref="C261" r:id="rId254" xr:uid="{8380DBBE-C42A-44E0-A990-3F6D492608A5}"/>
     <hyperlink ref="C262" r:id="rId255" xr:uid="{92C39D19-1599-44F9-8163-8F5DDB6B030A}"/>
+    <hyperlink ref="C263" r:id="rId256" xr:uid="{BBC6F217-70D0-41DC-B86E-2AE705EF915D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId256"/>
+  <pageSetup orientation="portrait" r:id="rId257"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: odd even Linked List
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB414A5C-E654-4F5F-B1AE-7868954A1DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94033200-73CC-4C7D-AFFB-648E1C344670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="528">
   <si>
     <t>date</t>
   </si>
@@ -1598,6 +1598,12 @@
   </si>
   <si>
     <t>find length of loop in Linked List</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/odd-even-linked-list/</t>
+  </si>
+  <si>
+    <t>odd even linked list</t>
   </si>
 </sst>
 </file>
@@ -1868,7 +1874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D263"/>
+  <dimension ref="A1:D264"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4760,6 +4766,17 @@
       </c>
       <c r="C263" s="4" t="s">
         <v>524</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A264" s="1">
+        <v>46220</v>
+      </c>
+      <c r="B264" t="s">
+        <v>527</v>
+      </c>
+      <c r="C264" s="4" t="s">
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -5020,8 +5037,9 @@
     <hyperlink ref="C261" r:id="rId254" xr:uid="{8380DBBE-C42A-44E0-A990-3F6D492608A5}"/>
     <hyperlink ref="C262" r:id="rId255" xr:uid="{92C39D19-1599-44F9-8163-8F5DDB6B030A}"/>
     <hyperlink ref="C263" r:id="rId256" xr:uid="{BBC6F217-70D0-41DC-B86E-2AE705EF915D}"/>
+    <hyperlink ref="C264" r:id="rId257" xr:uid="{1EA0E7FC-F8C6-4E61-993A-5E695914E17E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId257"/>
+  <pageSetup orientation="portrait" r:id="rId258"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: delete middle node of the linked list
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94033200-73CC-4C7D-AFFB-648E1C344670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1662DB31-7C25-43AA-90C9-B0E260ECBB7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="530">
   <si>
     <t>date</t>
   </si>
@@ -1604,6 +1604,12 @@
   </si>
   <si>
     <t>odd even linked list</t>
+  </si>
+  <si>
+    <t>delete the middle node of the linked list</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/delete-the-middle-node-of-a-linked-list/</t>
   </si>
 </sst>
 </file>
@@ -1874,7 +1880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D264"/>
+  <dimension ref="A1:D265"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4777,6 +4783,17 @@
       </c>
       <c r="C264" s="4" t="s">
         <v>526</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A265" s="1">
+        <v>46221</v>
+      </c>
+      <c r="B265" t="s">
+        <v>528</v>
+      </c>
+      <c r="C265" s="4" t="s">
+        <v>529</v>
       </c>
     </row>
   </sheetData>
@@ -5038,8 +5055,9 @@
     <hyperlink ref="C262" r:id="rId255" xr:uid="{92C39D19-1599-44F9-8163-8F5DDB6B030A}"/>
     <hyperlink ref="C263" r:id="rId256" xr:uid="{BBC6F217-70D0-41DC-B86E-2AE705EF915D}"/>
     <hyperlink ref="C264" r:id="rId257" xr:uid="{1EA0E7FC-F8C6-4E61-993A-5E695914E17E}"/>
+    <hyperlink ref="C265" r:id="rId258" xr:uid="{2355DF94-3ACD-4A6D-BCE3-6F0DF622A613}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId258"/>
+  <pageSetup orientation="portrait" r:id="rId259"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: sort LL containing 0, 1 and 2
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1662DB31-7C25-43AA-90C9-B0E260ECBB7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE33A36-1FA0-459D-9302-B29126238167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="532">
   <si>
     <t>date</t>
   </si>
@@ -1610,6 +1610,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/delete-the-middle-node-of-a-linked-list/</t>
+  </si>
+  <si>
+    <t>sort a linked list having 0s,1s and 2s</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/given-a-linked-list-of-0s-1s-and-2s-sort-it/1</t>
   </si>
 </sst>
 </file>
@@ -1880,7 +1886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D265"/>
+  <dimension ref="A1:D266"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4794,6 +4800,17 @@
       </c>
       <c r="C265" s="4" t="s">
         <v>529</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A266" s="1">
+        <v>46222</v>
+      </c>
+      <c r="B266" t="s">
+        <v>530</v>
+      </c>
+      <c r="C266" s="4" t="s">
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -5056,8 +5073,9 @@
     <hyperlink ref="C263" r:id="rId256" xr:uid="{BBC6F217-70D0-41DC-B86E-2AE705EF915D}"/>
     <hyperlink ref="C264" r:id="rId257" xr:uid="{1EA0E7FC-F8C6-4E61-993A-5E695914E17E}"/>
     <hyperlink ref="C265" r:id="rId258" xr:uid="{2355DF94-3ACD-4A6D-BCE3-6F0DF622A613}"/>
+    <hyperlink ref="C266" r:id="rId259" xr:uid="{159194C3-71FC-4692-8F5E-8E12E85D48C7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId259"/>
+  <pageSetup orientation="portrait" r:id="rId260"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: intersection point of 2 linked lists
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE33A36-1FA0-459D-9302-B29126238167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD60847B-F541-4B43-9704-C2452C5C5CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="534">
   <si>
     <t>date</t>
   </si>
@@ -1616,6 +1616,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/given-a-linked-list-of-0s-1s-and-2s-sort-it/1</t>
+  </si>
+  <si>
+    <t>find node where intersection happens in a y linked list</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
   </si>
 </sst>
 </file>
@@ -1886,7 +1892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D266"/>
+  <dimension ref="A1:D267"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4811,6 +4817,17 @@
       </c>
       <c r="C266" s="4" t="s">
         <v>531</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A267" s="1">
+        <v>46222</v>
+      </c>
+      <c r="B267" t="s">
+        <v>532</v>
+      </c>
+      <c r="C267" s="4" t="s">
+        <v>533</v>
       </c>
     </row>
   </sheetData>
@@ -5074,8 +5091,9 @@
     <hyperlink ref="C264" r:id="rId257" xr:uid="{1EA0E7FC-F8C6-4E61-993A-5E695914E17E}"/>
     <hyperlink ref="C265" r:id="rId258" xr:uid="{2355DF94-3ACD-4A6D-BCE3-6F0DF622A613}"/>
     <hyperlink ref="C266" r:id="rId259" xr:uid="{159194C3-71FC-4692-8F5E-8E12E85D48C7}"/>
+    <hyperlink ref="C267" r:id="rId260" xr:uid="{8B778C63-6102-480B-9DE3-84BD9B23CF17}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId260"/>
+  <pageSetup orientation="portrait" r:id="rId261"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: add 1 to no represeted as linked list
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD60847B-F541-4B43-9704-C2452C5C5CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D20C4C-CAEA-468A-BE67-E653FAF1C642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="536">
   <si>
     <t>date</t>
   </si>
@@ -1622,6 +1622,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/add-1-to-a-number-represented-as-linked-list/1</t>
+  </si>
+  <si>
+    <t>add 1 to a linked list</t>
   </si>
 </sst>
 </file>
@@ -1892,7 +1898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D267"/>
+  <dimension ref="A1:D268"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4828,6 +4834,17 @@
       </c>
       <c r="C267" s="4" t="s">
         <v>533</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A268" s="1">
+        <v>46222</v>
+      </c>
+      <c r="B268" t="s">
+        <v>535</v>
+      </c>
+      <c r="C268" s="4" t="s">
+        <v>534</v>
       </c>
     </row>
   </sheetData>
@@ -5092,8 +5109,9 @@
     <hyperlink ref="C265" r:id="rId258" xr:uid="{2355DF94-3ACD-4A6D-BCE3-6F0DF622A613}"/>
     <hyperlink ref="C266" r:id="rId259" xr:uid="{159194C3-71FC-4692-8F5E-8E12E85D48C7}"/>
     <hyperlink ref="C267" r:id="rId260" xr:uid="{8B778C63-6102-480B-9DE3-84BD9B23CF17}"/>
+    <hyperlink ref="C268" r:id="rId261" xr:uid="{D28C9BC5-5C24-460B-A590-6156856C591D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId261"/>
+  <pageSetup orientation="portrait" r:id="rId262"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: delete all occ of a key in DLL
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D20C4C-CAEA-468A-BE67-E653FAF1C642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DFC332-83C7-4893-B295-ABABE3A9645C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="538">
   <si>
     <t>date</t>
   </si>
@@ -1628,6 +1628,12 @@
   </si>
   <si>
     <t>add 1 to a linked list</t>
+  </si>
+  <si>
+    <t>delete all occurances of a given key in a DLL</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/delete-all-occurrences-of-a-given-key-in-a-doubly-linked-list/1</t>
   </si>
 </sst>
 </file>
@@ -1898,7 +1904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D268"/>
+  <dimension ref="A1:D269"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4845,6 +4851,17 @@
       </c>
       <c r="C268" s="4" t="s">
         <v>534</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A269" s="1">
+        <v>46223</v>
+      </c>
+      <c r="B269" t="s">
+        <v>536</v>
+      </c>
+      <c r="C269" s="4" t="s">
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -5110,8 +5127,9 @@
     <hyperlink ref="C266" r:id="rId259" xr:uid="{159194C3-71FC-4692-8F5E-8E12E85D48C7}"/>
     <hyperlink ref="C267" r:id="rId260" xr:uid="{8B778C63-6102-480B-9DE3-84BD9B23CF17}"/>
     <hyperlink ref="C268" r:id="rId261" xr:uid="{D28C9BC5-5C24-460B-A590-6156856C591D}"/>
+    <hyperlink ref="C269" r:id="rId262" xr:uid="{C32C105C-C331-4786-BFBC-C1321A242353}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId262"/>
+  <pageSetup orientation="portrait" r:id="rId263"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: find pairs with given sum in DLL and Remove duplicates from sorted DLL
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DFC332-83C7-4893-B295-ABABE3A9645C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63488AD-59B4-44AB-939C-4288C7B6ED53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="542">
   <si>
     <t>date</t>
   </si>
@@ -1634,6 +1634,18 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/delete-all-occurrences-of-a-given-key-in-a-doubly-linked-list/1</t>
+  </si>
+  <si>
+    <t>find pairs with given sum in DLL</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/find-pairs-with-given-sum-in-doubly-linked-list/1</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/remove-duplicates-from-a-sorted-doubly-linked-list/1</t>
+  </si>
+  <si>
+    <t>remove duplicates from a sorted DLL</t>
   </si>
 </sst>
 </file>
@@ -1904,7 +1916,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D269"/>
+  <dimension ref="A1:D271"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4862,6 +4874,28 @@
       </c>
       <c r="C269" s="4" t="s">
         <v>537</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A270" s="1">
+        <v>46223</v>
+      </c>
+      <c r="B270" t="s">
+        <v>538</v>
+      </c>
+      <c r="C270" s="4" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A271" s="1">
+        <v>46223</v>
+      </c>
+      <c r="B271" t="s">
+        <v>541</v>
+      </c>
+      <c r="C271" s="4" t="s">
+        <v>540</v>
       </c>
     </row>
   </sheetData>
@@ -5128,8 +5162,10 @@
     <hyperlink ref="C267" r:id="rId260" xr:uid="{8B778C63-6102-480B-9DE3-84BD9B23CF17}"/>
     <hyperlink ref="C268" r:id="rId261" xr:uid="{D28C9BC5-5C24-460B-A590-6156856C591D}"/>
     <hyperlink ref="C269" r:id="rId262" xr:uid="{C32C105C-C331-4786-BFBC-C1321A242353}"/>
+    <hyperlink ref="C270" r:id="rId263" xr:uid="{9F97A164-BAC7-4B68-B505-60450E954A4F}"/>
+    <hyperlink ref="C271" r:id="rId264" xr:uid="{15F7866B-4473-4A49-95A7-EDAE4B80D5A5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId263"/>
+  <pageSetup orientation="portrait" r:id="rId265"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem : Longest Bitonic Subsequence
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63488AD-59B4-44AB-939C-4288C7B6ED53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231B013C-FF73-42A2-AC4C-328C5DE9F258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="544">
   <si>
     <t>date</t>
   </si>
@@ -1646,6 +1646,12 @@
   </si>
   <si>
     <t>remove duplicates from a sorted DLL</t>
+  </si>
+  <si>
+    <t>Longest Bitonic Subsequence</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/longest-bitonic-subsequence0824/1</t>
   </si>
 </sst>
 </file>
@@ -1916,7 +1922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D271"/>
+  <dimension ref="A1:D272"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4896,6 +4902,17 @@
       </c>
       <c r="C271" s="4" t="s">
         <v>540</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A272" s="1">
+        <v>46225</v>
+      </c>
+      <c r="B272" t="s">
+        <v>542</v>
+      </c>
+      <c r="C272" s="4" t="s">
+        <v>543</v>
       </c>
     </row>
   </sheetData>
@@ -5164,8 +5181,9 @@
     <hyperlink ref="C269" r:id="rId262" xr:uid="{C32C105C-C331-4786-BFBC-C1321A242353}"/>
     <hyperlink ref="C270" r:id="rId263" xr:uid="{9F97A164-BAC7-4B68-B505-60450E954A4F}"/>
     <hyperlink ref="C271" r:id="rId264" xr:uid="{15F7866B-4473-4A49-95A7-EDAE4B80D5A5}"/>
+    <hyperlink ref="C272" r:id="rId265" xr:uid="{E899D1CC-DE6D-4F4A-957F-FF175B9D4760}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId265"/>
+  <pageSetup orientation="portrait" r:id="rId266"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Problem: count number of LIS
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Desktop\study_materials\DailyCPQuestionsPractise\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231B013C-FF73-42A2-AC4C-328C5DE9F258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D52155-9365-4F0D-B476-831DE0187B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="546">
   <si>
     <t>date</t>
   </si>
@@ -1652,6 +1652,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/longest-bitonic-subsequence0824/1</t>
+  </si>
+  <si>
+    <t>count number of LIS</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-longest-increasing-subsequence/</t>
   </si>
 </sst>
 </file>
@@ -1922,7 +1928,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D272"/>
+  <dimension ref="A1:D273"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" bestFit="1"/>
@@ -4913,6 +4919,17 @@
       </c>
       <c r="C272" s="4" t="s">
         <v>543</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A273" s="1">
+        <v>46226</v>
+      </c>
+      <c r="B273" t="s">
+        <v>544</v>
+      </c>
+      <c r="C273" s="4" t="s">
+        <v>545</v>
       </c>
     </row>
   </sheetData>
@@ -5182,8 +5199,9 @@
     <hyperlink ref="C270" r:id="rId263" xr:uid="{9F97A164-BAC7-4B68-B505-60450E954A4F}"/>
     <hyperlink ref="C271" r:id="rId264" xr:uid="{15F7866B-4473-4A49-95A7-EDAE4B80D5A5}"/>
     <hyperlink ref="C272" r:id="rId265" xr:uid="{E899D1CC-DE6D-4F4A-957F-FF175B9D4760}"/>
+    <hyperlink ref="C273" r:id="rId266" xr:uid="{6C8F2F70-18CC-4A18-B5CA-CF7E77991D2E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId266"/>
+  <pageSetup orientation="portrait" r:id="rId267"/>
 </worksheet>
 </file>
</xml_diff>